<commit_message>
finalized stucture and moved data to excel sheet, fixed increase decrease c7 injection
</commit_message>
<xml_diff>
--- a/statics/static_sheet.xlsx
+++ b/statics/static_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UTHIHI\PycharmProjects\MoamProject\statics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BABDABE2-F9F7-42AA-96C1-5B9A10792E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B415B3D-02D8-4E1B-832C-F7E0DFC8A124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{BEDCD23D-130C-4D40-8649-08CA7512DBD5}"/>
+    <workbookView xWindow="28680" yWindow="1620" windowWidth="29040" windowHeight="17520" xr2:uid="{BEDCD23D-130C-4D40-8649-08CA7512DBD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmarks" sheetId="4" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="266">
   <si>
     <t>BENCHMARK ID</t>
   </si>
@@ -840,6 +840,15 @@
   </si>
   <si>
     <t>https://www.vanlanschotkempen.com/-/media/files/documents/corporate/investor-relations-en/debt-investors/library/dip/2025/prospectus/securities-note---15-may-2025.ashx</t>
+  </si>
+  <si>
+    <t>IGV US</t>
+  </si>
+  <si>
+    <t>iShares Expanded Tech-Software Sector ETF</t>
+  </si>
+  <si>
+    <t>US Software</t>
   </si>
 </sst>
 </file>
@@ -965,7 +974,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -991,6 +1000,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1348,7 +1359,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69353C34-D752-4EE8-9624-BFD9BF9C419E}">
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -1980,6 +1991,17 @@
       </c>
       <c r="E58" t="s">
         <v>230</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D59" t="s">
+        <v>264</v>
+      </c>
+      <c r="E59" t="s">
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -2227,7 +2249,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD660241-4EC6-4BC1-A445-D102A6866814}">
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -2531,6 +2553,14 @@
         <v>21</v>
       </c>
       <c r="B38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="19" t="s">
+        <v>263</v>
+      </c>
+      <c r="B39" s="20">
         <v>3</v>
       </c>
     </row>

</xml_diff>